<commit_message>
feat(core): universalizacao multi-obras completa dos 13 motores e higienizacao de scripts
- Transforma todos os scripts python em motores universais com CLI (--obra e --dir)
- Desacopla 100% dos dados de obras (config_obra.json, titulos_desenhos.json, catalogos)
- Cria estrutura modelo projetos/_TEMPLATE_OBRA_NOVA/ com guia de onboarding
- Higieniza raiz de scripts/, movendo legados e wrappers para scripts/_legado_tmult/
- Atualiza governanca em agents.md e SKILL_DEV_SENIOR.md com regra mandatoria multi-obras
- Valida nao-regressao na OBRA_TMULT (158 itens, R$ 1.660.762,28) e teste no RESIDENCIAL_ALPHA
</commit_message>
<xml_diff>
--- a/projetos/OBRA_TMULT/02_ORCAMENTO_BASE_E_CONTRATOS/CURVA_ABC_SERVICOS_E_INSUMOS_TMULT.xlsx
+++ b/projetos/OBRA_TMULT/02_ORCAMENTO_BASE_E_CONTRATOS/CURVA_ABC_SERVICOS_E_INSUMOS_TMULT.xlsx
@@ -582,7 +582,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CURVA ABC DE FAMÍLIAS DE INSUMOS &amp; RECURSOS — OBRA TMULT</t>
+          <t>CURVA ABC DE FAMÍLIAS DE INSUMOS &amp; RECURSOS — TMULT</t>
         </is>
       </c>
     </row>
@@ -590,7 +590,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Abertura Analítica do Custo Direto Total: R$ 1,129,722.67 | Base SINAPI SP 07/2026</t>
+          <t>Abertura Analítica do Custo Direto Total: R$ 1,129,722.67</t>
         </is>
       </c>
     </row>

</xml_diff>